<commit_message>
Expand test cases to 50 across 5 sheets
</commit_message>
<xml_diff>
--- a/selenium-tests/BookSphere_TestCases.xlsx
+++ b/selenium-tests/BookSphere_TestCases.xlsx
@@ -519,17 +519,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -538,7 +538,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BookSphere — Login Tests Test Cases</t>
+          <t>BookSphere — Login Tests  (14 Test Cases)</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>TC_L_01</t>
@@ -637,7 +637,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>User is redirected to catalog/home page after successful login</t>
+          <t>User redirected to catalog/home page</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -657,7 +657,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC_L_02</t>
@@ -670,7 +670,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Wrong password shows error</t>
+          <t>Wrong password shows lf-error-msg</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Error message displayed below form (class: lf-error-msg)</t>
+          <t>Error message (class: lf-error-msg) appears below form</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -713,7 +713,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TC_L_03</t>
@@ -726,7 +726,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Empty email field — inline validation</t>
+          <t>Empty email — inline field validation</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>'Enter a valid email' error shown under email field</t>
+          <t>'Enter a valid email' error under email field (lf-err-msg)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -765,7 +765,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>TC_L_04</t>
@@ -778,7 +778,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Empty password field — inline validation</t>
+          <t>Empty password — inline field validation</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>'Password is required' error shown under password field</t>
+          <t>'Password is required' shown under password field</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
@@ -817,7 +817,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="7" ht="58" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TC_L_05</t>
@@ -869,7 +869,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="52" customHeight="1">
+    <row r="8" ht="58" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>TC_L_06</t>
@@ -882,7 +882,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Password toggle show/hide</t>
+          <t>Password show/hide toggle</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -893,10 +893,10 @@
       <c r="E8" s="3" t="inlineStr">
         <is>
           <t>1. Enter password: Varad@999
-2. Click 👁️ icon
-3. Verify password is visible
-4. Click 🙈 icon
-5. Verify password is masked</t>
+2. Click 👁️ button
+3. Verify type=text
+4. Click 🙈 button
+5. Verify type=password</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Password toggles between text and password type</t>
+          <t>Input type toggles between text and password</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
@@ -922,7 +922,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="52" customHeight="1">
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>TC_L_07</t>
@@ -935,7 +935,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Switch to Sign Up mode</t>
+          <t>Switch to Sign Up mode shows Name field</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -946,7 +946,7 @@
       <c r="E9" s="3" t="inlineStr">
         <is>
           <t>1. Click 'Sign Up' toggle button
-2. Verify form now shows Full Name field</t>
+2. Verify Full Name field appears</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Form switches to register mode, Full Name field appears</t>
+          <t>Form switches to register mode, Full Name input visible</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -972,7 +972,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="52" customHeight="1">
+    <row r="10" ht="58" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>TC_L_08</t>
@@ -985,7 +985,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Forgot password flow</t>
+          <t>Forgot password sends reset email</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         <is>
           <t>1. Enter email: varadmandhare924@gmail.com
 2. Click 'Forgot password?'
-3. Verify success message</t>
+3. Check success message</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>'✓ Reset link sent to varadmandhare924@gmail.com' shown</t>
+          <t>'✓ Reset link sent to varadmandhare924@gmail.com' visible</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="58" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>TC_L_09</t>
@@ -1046,9 +1046,9 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>1. Login successfully
-2. Refresh the browser (F5)
-3. Check if user stays logged in</t>
+          <t>1. Login with valid credentials
+2. Refresh browser (F5)
+3. Verify still on catalog</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>User remains on catalog page — not redirected to login</t>
+          <t>User stays on catalog — not redirected to login</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -1070,6 +1070,267 @@
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TC_L_10</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Both fields empty — both errors shown</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>User on login page</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>1. Leave email and password both blank
+2. Click 'Sign In →'</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Email: (empty)
+Password: (empty)</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Validation errors shown under both email and password fields</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>TC_L_11</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>SQL injection in email field is rejected</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>User on login page</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>1. Enter email: ' OR '1'='1
+2. Enter password: Varad@999
+3. Click 'Sign In →'</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Email: ' OR '1'='1
+Password: Varad@999</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Validation error shown — login does not succeed, no crash</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>TC_L_12</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Very long email string handled gracefully</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>User on login page</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>1. Enter 300-character string as email
+2. Click 'Sign In →'</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Email: aaa...@bbb.com (300 chars)
+Password: Varad@999</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Form validates / shows error — no crash or unhandled exception</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TC_L_13</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Register new account with valid data</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>User on login page in Sign Up mode</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>1. Click 'Sign Up' toggle
+2. Enter name: Test User
+3. Enter email: newtestuser99@gmail.com
+4. Enter password: Test@1234
+5. Click 'Create Account →'</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Name: Test User
+Email: newtestuser99@gmail.com
+Password: Test@1234</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Success message shown: 'Account created! Signing you in…'</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>TC_L_14</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Register with weak password &lt; 6 chars</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>User in Sign Up mode</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>1. Click 'Sign Up' toggle
+2. Enter name, email
+3. Enter password: 123
+4. Click 'Create Account →'</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Password: 123 (3 chars)</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>'Minimum 6 characters' error shown under password field</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
@@ -1089,17 +1350,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -1108,7 +1369,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BookSphere — Catalog Tests Test Cases</t>
+          <t>BookSphere — Catalog Tests  (12 Test Cases)</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1430,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>TC_C_01</t>
@@ -1182,7 +1443,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>All books load on catalog page</t>
+          <t>All 12 books load on catalog page</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1194,7 +1455,7 @@
         <is>
           <t>1. Login successfully
 2. Navigate to catalog page
-3. Count book cards displayed</t>
+3. Count product-card elements</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -1204,7 +1465,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>12 book cards are displayed</t>
+          <t>12 book cards rendered on page</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -1220,7 +1481,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC_C_02</t>
@@ -1243,7 +1504,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>1. Type 'Atomic' in the search input
+          <t>1. Type 'Atomic' in search input
 2. Observe filtered results</t>
         </is>
       </c>
@@ -1254,7 +1515,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Only books matching 'Atomic' tag/title are shown (≥1 result, fewer than total)</t>
+          <t>≥1 result shown, fewer cards than total 12</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -1270,7 +1531,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TC_C_03</t>
@@ -1283,7 +1544,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Search by author name</t>
+          <t>Search by author name — James Clear</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1293,8 +1554,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1. Type author name in search input
-2. Observe results</t>
+          <t>1. Type 'James Clear' in search input</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1304,7 +1564,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Books by James Clear appear in results</t>
+          <t>Books by James Clear shown in results</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -1320,7 +1580,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>TC_C_04</t>
@@ -1333,7 +1593,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Search returns no results for garbage input</t>
+          <t>Search by tag — 'classic'</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1343,17 +1603,18 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1. Type 'xyzxyzxyz' in search input</t>
+          <t>1. Type 'classic' in search input
+2. Check results</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Search query: xyzxyzxyz</t>
+          <t>Search query: classic</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Empty state / no books shown — no crash</t>
+          <t>Books tagged 'classic' are shown</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
@@ -1369,7 +1630,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="7" ht="58" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TC_C_05</t>
@@ -1382,7 +1643,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Genre tree is visible</t>
+          <t>Search returns empty state for garbage input</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1392,33 +1653,33 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1. Look for genre/category tree on the page</t>
+          <t>1. Type 'xyzxyzxyz' in search input</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Search query: xyzxyzxyz</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Genre tree nodes are visible and rendered</t>
+          <t>No books shown, empty state displayed — no crash</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Smoke</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>TC_C_06</t>
@@ -1431,28 +1692,29 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Click genre node filters books</t>
+          <t>Clear search restores full catalog</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>User on catalog page, genre tree visible</t>
+          <t>User on catalog page, search active</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>1. Click on a genre node (e.g. Fiction)
-2. Observe books shown</t>
+          <t>1. Type 'Atomic' in search
+2. Clear the search input
+3. Count books again</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Genre: Fiction</t>
+          <t>Search query cleared</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Only books under Fiction category are displayed</t>
+          <t>All 12 books shown again after clearing search</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
@@ -1468,7 +1730,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="52" customHeight="1">
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>TC_C_07</t>
@@ -1481,7 +1743,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Price sort — Low to High</t>
+          <t>Genre tree is visible and rendered</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1491,28 +1753,277 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>1. Select 'Price: Low to High' sort option
-2. Check order of displayed prices</t>
+          <t>1. Check for genre tree nodes (.tree-node)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Sort: Price ascending</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Books displayed in ascending order of price</t>
+          <t>Genre tree nodes visible on the page</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="3" t="inlineStr">
         <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>TC_C_08</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Click Fiction genre filters books</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Genre tree visible</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>1. Click 'Fiction' genre node
+2. Observe book cards</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Genre: Fiction</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Only Fiction books displayed</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TC_C_09</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Price sort — Low to High</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>User on catalog page</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>1. Select 'Price: Low to High' sort
+2. Read first and last book price</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Sort: price ascending</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>First book has lowest price, last has highest</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TC_C_10</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Price sort — High to Low</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>User on catalog page</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>1. Select 'Price: High to Low' sort
+2. Read first and last book price</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Sort: price descending</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>First book has highest price, last has lowest</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>TC_C_11</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Book card shows title, author, price</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>User on catalog page</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>1. Look at any book card
+2. Verify title, author and price are visible</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Each card displays title, author name and price (₹)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>TC_C_12</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Add to Wishlist from catalog</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>User logged in, on catalog page</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>1. Click wishlist/heart icon on any book
+2. Navigate to Wishlist page</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Book appears in Wishlist page (HashSet — no duplicates)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
@@ -1532,17 +2043,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -1551,7 +2062,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BookSphere — Cart Tests Test Cases</t>
+          <t>BookSphere — Cart Tests  (12 Test Cases)</t>
         </is>
       </c>
     </row>
@@ -1612,7 +2123,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>TC_CA_01</t>
@@ -1625,7 +2136,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Add book to cart</t>
+          <t>Add book to cart from catalog</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1646,7 +2157,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Cart page shows at least 1 item</t>
+          <t>Cart page shows ≥1 item</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -1662,7 +2173,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC_CA_02</t>
@@ -1675,19 +2186,19 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Remove item from cart</t>
+          <t>Cart item count updates in navbar</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Cart has at least 1 item</t>
+          <t>User on catalog page</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>1. Go to cart
-2. Click remove button on first item
-3. Verify item is gone</t>
+          <t>1. Note cart count in navbar
+2. Add a book to cart
+3. Check navbar count again</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1697,7 +2208,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Item is removed from cart, count decreases by 1</t>
+          <t>Navbar cart counter increments by 1</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -1713,7 +2224,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TC_CA_03</t>
@@ -1726,139 +2237,138 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Undo remove restores item (Stack DSA)</t>
+          <t>Add same book twice — quantity increases</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Cart has at least 1 item</t>
+          <t>User on catalog page</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>1. Add the same book to cart twice
+2. Go to cart
+3. Check qty for that book</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Same book added twice</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Quantity shows 2 for that book (not two separate rows)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>TC_CA_04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Remove item from cart</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Cart has ≥1 item</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>1. Go to /cart
+2. Click remove (✕) on first item
+3. Verify item gone</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Item removed, cart count decreases by 1</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>TC_CA_05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Undo remove restores item — Stack DSA</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Cart has ≥1 item</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>1. Remove an item
 2. Click 'Undo' button
 3. Check item count</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Removed item is restored — cart count goes back to original</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>TC_CA_04</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Cart</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Apply coupon BOOK30</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Cart has items, total ≥ ₹200</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>1. Enter coupon code: BOOK30
-2. Click Apply
-3. Check discount shown</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Coupon: BOOK30
-Min spend: ₹200</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>₹30 discount is applied and shown on cart total</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>TC_CA_05</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Cart</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Apply coupon BOOK80</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Cart total ≥ ₹500</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>1. Enter coupon: BOOK80
-2. Click Apply</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Coupon: BOOK80
-Min spend: ₹500</t>
-        </is>
-      </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>₹80 discount applied</t>
+          <t>Removed item restored — count back to original (Stack LIFO)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1867,7 +2377,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="52" customHeight="1">
+    <row r="8" ht="58" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>TC_CA_06</t>
@@ -1880,44 +2390,45 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Invalid coupon shows error</t>
+          <t>Undo button disappears after cart empty</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Cart has items</t>
+          <t>Cart has 1 item</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>1. Enter coupon: FAKECODE
-2. Click Apply</t>
+          <t>1. Remove the only item
+2. Undo it
+3. Remove again — verify no undo visible after fresh load</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Coupon: FAKECODE</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Error or no discount applied — not crashes</t>
+          <t>Undo only available when stack has items</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="52" customHeight="1">
+          <t>Functional</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>TC_CA_07</t>
@@ -1930,28 +2441,31 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Place standard order</t>
+          <t>Apply coupon BOOK30 — min spend ₹200</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Cart has items, user logged in</t>
+          <t>Cart total ≥ ₹200</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>1. Click 'Place Order'
-2. Navigate to Orders page</t>
+          <t>1. Enter coupon: BOOK30
+2. Click Apply
+3. Check discount row</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Coupon: BOOK30
+Min spend: ₹200
+Discount: ₹30</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Order appears on Orders page with PENDING status</t>
+          <t>₹30 discount shown, total reduced by ₹30</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -1962,6 +2476,262 @@
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>TC_CA_08</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Apply coupon BOOK80 — min spend ₹500</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Cart total ≥ ₹500</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>1. Enter coupon: BOOK80
+2. Click Apply</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Coupon: BOOK80
+Min spend: ₹500
+Discount: ₹80</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>₹80 discount applied</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TC_CA_09</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Apply coupon BOOK150 — min spend ₹900</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Cart total ≥ ₹900</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>1. Enter coupon: BOOK150
+2. Click Apply</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Coupon: BOOK150
+Min spend: ₹900
+Discount: ₹150</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>₹150 discount applied</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TC_CA_10</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Apply invalid coupon shows no discount</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Cart has items</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>1. Enter coupon: FAKECODE
+2. Click Apply</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Coupon: FAKECODE</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>No discount applied, error or empty state shown — no crash</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>TC_CA_11</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Discount engine — DP picks best combination</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Cart total ≥ ₹900, all coupons available</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>1. Add books worth ≥ ₹900
+2. Let DP engine auto-select best coupons
+3. Verify discount is optimal</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Total ≥ ₹900
+Best combo: BOOK30 + BOOK80 + BOOK150 = ₹260</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>DP selects maximum discount without exceeding budget (0/1 Knapsack)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>TC_CA_12</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Place standard order clears cart</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Cart has items, user logged in</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>1. Click 'Place Order'
+2. Go back to cart</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Cart is empty after order placed, order appears in Orders page</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
@@ -1981,17 +2751,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -2000,7 +2770,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BookSphere — Orders Tests Test Cases</t>
+          <t>BookSphere — Orders Tests  (7 Test Cases)</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2831,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>TC_O_01</t>
@@ -2079,13 +2849,13 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>User has placed at least one order</t>
+          <t>User has placed ≥1 order</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>1. Navigate to /orders
-2. Count order cards</t>
+2. Check order cards visible</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -2095,7 +2865,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Order cards are displayed</t>
+          <t>Order cards rendered on the page</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -2111,7 +2881,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC_O_02</t>
@@ -2124,19 +2894,20 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Premium order appears first (Priority Queue DSA)</t>
+          <t>Premium order appears first — Priority Queue DSA</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>User is premium, has placed premium + standard orders</t>
+          <t>User is premium, has both premium and standard orders</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>1. Place a premium order
-2. Go to Orders page
-3. Check order of cards</t>
+          <t>1. Place premium order (priority=1)
+2. Place standard order (priority=10)
+3. Go to Orders page
+4. Check order of cards</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -2146,7 +2917,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Premium order (priority=1) appears before standard (priority=10)</t>
+          <t>Premium order (priority=1) listed above standard (priority=10)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -2162,7 +2933,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TC_O_03</t>
@@ -2175,7 +2946,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Order status shows PENDING after placement</t>
+          <t>New order status shows PENDING</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2186,8 +2957,8 @@
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>1. Place order
-2. Go to Orders page
-3. Check status label</t>
+2. Navigate to /orders
+3. Check status badge</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -2197,7 +2968,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Status badge shows PENDING</t>
+          <t>Status badge shows 'PENDING'</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -2210,6 +2981,212 @@
       <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>TC_O_04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Order contains correct book items and total</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Order placed with specific books</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>1. Add book (₹599) to cart
+2. Place order
+3. Open order on Orders page
+4. Verify item name and total</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Book: The Pragmatic Programmer ₹599</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Order shows correct book name, qty and total amount</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>TC_O_05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Multiple orders are all listed</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>User has placed 3+ orders</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>1. Place 3 separate orders
+2. Navigate to /orders
+3. Count order cards</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>All 3 orders visible on the page</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TC_O_06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Orders sorted by priority — premium always first</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Multiple orders with different priorities</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1. Place standard order
+2. Place premium order
+3. Go to /orders
+4. Verify sort order</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Standard priority=10
+Premium priority=1</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Orders sorted ascending by priority — premium (1) before standard (10)</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>TC_O_07</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Empty orders page shows empty state</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>User with no orders placed</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>1. Log in as new user with no orders
+2. Navigate to /orders</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>No prior orders</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Empty state message shown — no errors, no blank white screen</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
         </is>
       </c>
     </row>
@@ -2230,14 +3207,14 @@
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -2246,7 +3223,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BookSphere — API Tests Test Cases</t>
+          <t>BookSphere — API Tests  (5 Test Cases)</t>
         </is>
       </c>
     </row>
@@ -2307,7 +3284,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>TC_A_01</t>
@@ -2320,28 +3297,29 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>GET /books returns 200</t>
+          <t>GET /books returns 200 with 12 books</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Valid anon key available</t>
+          <t>Valid anon key configured in ApiTest.java</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>1. Send GET to /rest/v1/books?select=*
-2. Include apikey header</t>
+          <t>1. Send GET /rest/v1/books?select=*
+2. Include apikey header
+3. Check status code and body</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>apikey: sb_publishable_5pi0OY09...</t>
+          <t>apikey: sb_publishable_5pi0OY09IbihgQliazw5ug_G5ha_SxJ</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200, JSON array of 12 books</t>
+          <t>HTTP 200, JSON array with 12 book objects</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -2357,7 +3335,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC_A_02</t>
@@ -2370,7 +3348,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>GET /coupons returns 200</t>
+          <t>GET /coupons returns 200 with 4 coupons</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -2380,7 +3358,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>1. Send GET to /rest/v1/coupons?select=*
+          <t>1. Send GET /rest/v1/coupons?select=*
 2. Include apikey header</t>
         </is>
       </c>
@@ -2391,7 +3369,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200, JSON array of 4 coupons</t>
+          <t>HTTP 200, JSON array with 4 coupon objects (BOOK30/80/150/300)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -2407,7 +3385,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TC_A_03</t>
@@ -2420,7 +3398,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>GET /books filtered by category</t>
+          <t>GET /books filtered by category=Fiction returns 200</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2430,7 +3408,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1. Send GET to /rest/v1/books?select=*&amp;category=eq.Fiction</t>
+          <t>1. Send GET /rest/v1/books?select=*&amp;category=eq.Fiction</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -2440,7 +3418,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200, only Fiction books returned</t>
+          <t>HTTP 200, only Fiction category books in response</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -2456,7 +3434,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>TC_A_04</t>
@@ -2469,7 +3447,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>GET /books sorted by price</t>
+          <t>GET /books sorted by price ascending returns 200</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -2479,7 +3457,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1. Send GET to /rest/v1/books?select=*&amp;order=price.asc</t>
+          <t>1. Send GET /rest/v1/books?select=*&amp;order=price.asc</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -2489,7 +3467,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200, books in ascending price order</t>
+          <t>HTTP 200, books ordered by price lowest first</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
@@ -2505,7 +3483,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="7" ht="58" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TC_A_05</t>
@@ -2518,28 +3496,29 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>GET /carts without JWT returns 401</t>
+          <t>GET /carts without JWT returns 401 — RLS enforced</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>No JWT token provided</t>
+          <t>No Authorization header sent</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1. Send GET to /rest/v1/carts?select=*
-2. Only include apikey, no Authorization header</t>
+          <t>1. Send GET /rest/v1/carts?select=*
+2. Include only apikey header
+3. No Authorization header</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>No Authorization header</t>
+          <t>Authorization header: missing</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>HTTP 401 — private endpoint blocked</t>
+          <t>HTTP 401 — Supabase RLS blocks unauthenticated access to private table</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>

</xml_diff>